<commit_message>
add source and destination spot buy in controller and all blade files
Tracking view fixed in blade file, update spot buy xls file to add Source Code and Destination code
</commit_message>
<xml_diff>
--- a/public/consignmentapp_SampleDATA/spotby.xlsx
+++ b/public/consignmentapp_SampleDATA/spotby.xlsx
@@ -16,13 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
-  <si>
-    <t>From</t>
-  </si>
-  <si>
-    <t>To</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Vehicle Type</t>
   </si>
@@ -57,12 +51,6 @@
   </si>
   <si>
     <t>RFQ END Date &amp; Time</t>
-  </si>
-  <si>
-    <t>Ahmedabad</t>
-  </si>
-  <si>
-    <t>Aligarh</t>
   </si>
   <si>
     <t>2210CBT</t>
@@ -98,6 +86,12 @@
   </si>
   <si>
     <t>Closed body truck only</t>
+  </si>
+  <si>
+    <t>SourceCode</t>
+  </si>
+  <si>
+    <t>DestinationCode</t>
   </si>
 </sst>
 </file>
@@ -511,6 +505,7 @@
   <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="2" max="2" width="18.1796875" customWidth="1"/>
     <col min="9" max="9" width="17.1796875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.36328125" customWidth="1"/>
     <col min="11" max="11" width="17.90625" customWidth="1"/>
@@ -519,60 +514,60 @@
   <sheetData>
     <row r="1" spans="1:13" ht="39" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="4">
+        <v>5513</v>
+      </c>
+      <c r="B2" s="5">
+        <v>5704</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>13</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="F2" s="5">
         <v>2</v>
@@ -581,7 +576,7 @@
         <v>650</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I2" s="5">
         <v>15</v>
@@ -590,7 +585,7 @@
         <v>10</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L2" s="8">
         <v>45907.397048611114</v>

</xml_diff>